<commit_message>
Ajustes - Pendientes: Ajustar opciones Lambdatest Automatizado MAC & ANDROID no detectan la opción elegida al usar Programado test, Email se envía aún si se destilda opción fix pendiente. Sumar apartado design & funcionalidad programado test, de weekly
</commit_message>
<xml_diff>
--- a/data/Lead_information_Formulario_Bolivia_Main.xlsx
+++ b/data/Lead_information_Formulario_Bolivia_Main.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,11 @@
           <t>https://secure-developments.com/commonwealth/bolivia/gm_front/form/model-overviews?model=suburban</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>suburban</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Natalia</t>
@@ -520,48 +524,6 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://www.chevrolet.com.bo/solicitar-cotizacion</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://secure-developments.com/commonwealth/bolivia/gm_admin/form/raq</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Romina Monica</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Ibáñez</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>16343149</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>69077337</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>rominamonicaibanez_bo47@mrm.com</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
OverlayAjuste - Email ajuste reporte incluidas las urls insertas
</commit_message>
<xml_diff>
--- a/data/Lead_information_Formulario_Bolivia_Main.xlsx
+++ b/data/Lead_information_Formulario_Bolivia_Main.xlsx
@@ -492,27 +492,27 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ignacio Florencia</t>
+          <t>Gonzalo</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fuentes Flores</t>
+          <t>Salazar</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>35563922</t>
+          <t>16530879</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>66794464</t>
+          <t>74074395</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ignacioflorenciafuentesflores.bo28@mrm.com</t>
+          <t>gonzalosalazar_bo54@mrm.com</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -523,38 +523,38 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.chevrolet.com.bo/autos/onix</t>
+          <t>https://www.chevrolet.com.bo/suvs/suburban</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://secure-developments.com/commonwealth/bolivia/gm_front/form/model-overviews?model=onix</t>
+          <t>https://secure-developments.com/commonwealth/bolivia/gm_front/form/model-overviews?model=suburban</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Susana Rafael</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Perez Acosta</t>
+          <t>Gutierrez Serrano</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>86475769</t>
+          <t>13745287</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>78636469</t>
+          <t>61245914</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>susanarafaelperezacosta_bo85@mrm.com</t>
+          <t>sofiagutierrezserrano_bo34@mrm.com</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -570,33 +570,33 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://secure-developments.com/commonwealth/bolivia/gm_admin/form/raq</t>
+          <t>https://secure-developments.com/commonwealth/bolivia/gm_front/form/raq</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Matías Luis</t>
+          <t>Nicolás</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mendoza</t>
+          <t>Lopez Bravo</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>94696797</t>
+          <t>36494659</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>61224513</t>
+          <t>70608301</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>matiasluismendoza.bo50@mrm.com</t>
+          <t>nicolaslopezbravo.bo34@mrm.com</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>

</xml_diff>